<commit_message>
docs: add NW onboarding/add-flow Sr-UI-Designer review items (group F) to master list
UI-1..9: the 6-point add-flow critique + setup-flow recommendations, status-verified —
DONE: default-taxable+account-first, quick-add/smart-defaults, donut=allocation labeling,
total-value bond form. PARTIAL: one-reused-+Add (chose smart per-section), warmer tone,
recap-hub. OPEN: Finish success moment, setup-choice one-way door.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-master-action-list-2026-06-28.xlsx
+++ b/docs/finwise-master-action-list-2026-06-28.xlsx
@@ -477,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K39"/>
+  <dimension ref="A1:K49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1682,7 +1682,7 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>— D. PARKED V1 — launch blockers (see finwise-launch-and-parked.xlsx) —</t>
+          <t>— F. NW ONBOARDING / ADD-FLOW — my Sr UI Designer review (earlier this session) —</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr"/>
@@ -1699,47 +1699,47 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>L-1</t>
+          <t>UI-1</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Net Worth</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Switch to a paid/licensed price source (Tiingo). Free Yahoo feed isn't legal for a paid app</t>
+          <t>Wrapper question over-asked for the common taxable case; class-first fought the account-first mental model</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Parked V1</t>
+          <t>Sr UI Designer review</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>Seam ready; needs your API key</t>
+          <t>Add picker defaults wrapper='Taxable' + offers account-first picks (Retirement / Brokerage)</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>You get a key; I do the swap</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr"/>
@@ -1748,47 +1748,47 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>P-71</t>
+          <t>UI-2</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Branding</t>
+          <t>Net Worth</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Pick + trademark final app name ('FinWise' may be taken; 'Hatcho' front-runner)</t>
+          <t>Step-count fatigue in the add flow</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Parked V1</t>
+          <t>Sr UI Designer review</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Quick-add row + smart defaults + smart per-section jump (NW-12)</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>Decide name; then I do the rename pass (once, late)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr"/>
@@ -1797,47 +1797,47 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>L-5..L-26</t>
+          <t>UI-3</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Launch ops</t>
+          <t>Net Worth</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>App Store listing, privacy questionnaire, reviewer login, screenshots, build #35, submit</t>
+          <t>7 icon-only 'add more' buttons + 3 overlapping entry points → I'd recommended ONE reused '+ Add an account'</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Parked V1</t>
+          <t>Sr UI Designer review</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Blocker</t>
-        </is>
-      </c>
-      <c r="F30" s="6" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>Your-owned; build #35 blocked on free EAS quota (~Jul 1)</t>
+          <t>Chose smart per-section +Add (4 contextual buttons) instead of ONE; the single setup-hub button wasn't built</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>Sequence after the code is launch-ready</t>
+          <t>DECIDE: keep smart per-section (current) OR collapse to one '+ Add an account'. Your call</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr"/>
@@ -1846,113 +1846,145 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>P-23/P-63</t>
+          <t>UI-4</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Net Worth</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Dependency security scan + audit all data-fetch error handling (not just happy path)</t>
+          <t>View-by-section vs add-by-class mismatch confused the model</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Parked V1</t>
+          <t>Sr UI Designer review</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Important</t>
-        </is>
-      </c>
-      <c r="F31" s="6" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Captions label donut = allocation, sections = accounts (NW-8)</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>I can do both before submit</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr"/>
       <c r="K31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>— E. PARKED — fast-follow &amp; V2 highlights (full list in parked xlsx) —</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
-      <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>UI-5</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Net Worth</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Heavy individual-bond form deterred entry</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Sr UI Designer review</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Bonds form takes a total value + 'Add specific holdings →' link (NW-16)</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr"/>
+      <c r="K32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>P-1</t>
+          <t>UI-6</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Net Worth</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Bank/brokerage linking (auto-sync balances &amp; transactions)</t>
+          <t>Cold tone → wanted net-worth-as-hero + gentle nudges + warmer coaching voice</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>Parked V2</t>
+          <t>Sr UI Designer review</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
-        </is>
-      </c>
-      <c r="F33" s="6" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>Large build; needs secure server</t>
+          <t>Donut/net-worth hero + mixed-allocation nudge exist; warmer copy + celebratory moments not done</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>SEE PM REVIEW — this is the #1 retention lever; reconsider priority</t>
+          <t>Do a coaching-tone copy pass + add a success moment (see UI-8)</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="J33" s="5" t="inlineStr"/>
@@ -1961,22 +1993,22 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>P-8</t>
+          <t>UI-7</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Insights</t>
+          <t>Net Worth</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>'Can I afford a $600k house?' — plain-question affordability simulator</t>
+          <t>Setup flow: the polished recap/hub ('net worth so far' + '+ Add' + "I'm done") with net-worth-as-hero</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Parked V2</t>
+          <t>Sr UI Designer review / approved mock</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -1984,19 +2016,19 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="F34" s="6" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>Not built</t>
+          <t>Guided wizard shows a running 'Net worth so far' + Finish, but the polished recap-hub mock was never built as designed</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>SEE PM REVIEW — standout/shareable; move up</t>
+          <t>Build the recap-hub, OR confirm the current wizard is enough</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
@@ -2010,27 +2042,27 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>P-35</t>
+          <t>UI-8</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>UI/UX</t>
+          <t>Net Worth</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Home card: net worth over time ('up $40k in 6 months')</t>
+          <t>Guided 'Finish' has no success/celebration moment — anticlimactic after a multi-step setup</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Parked V2</t>
+          <t>Sr UI Designer review + NW audit</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -2040,12 +2072,12 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>Snapshot only today</t>
+          <t>NetWorthScreen: Finish → setNwSetupChoice('self'), no confirmation</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr">
         <is>
-          <t>SEE PM REVIEW — retention dopamine; move up</t>
+          <t>Add a 'You're set — here's your net worth' beat</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
@@ -2059,27 +2091,27 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>P-53</t>
+          <t>UI-9</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Goals</t>
+          <t>Net Worth</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Finish the full savings-goals screen (progress, priority, projections)</t>
+          <t>Setup choice is a one-way door — can't return to the guided walkthrough after picking 'I'll add my own'</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Parked fast-follow</t>
+          <t>Sr UI Designer review + NW audit</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>UX</t>
         </is>
       </c>
       <c r="F36" s="6" t="inlineStr">
@@ -2089,95 +2121,63 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>Logic exists; visual screen unfinished</t>
+          <t>nwSetupChoice can't be reset from the UI</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr">
         <is>
-          <t>Good stickiness; pair with OPEN-3</t>
+          <t>Add a way to re-enter guided setup (e.g. from a menu / Settings)</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr"/>
       <c r="K36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
-        <is>
-          <t>P-28/P-29</t>
-        </is>
-      </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>a11y</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Screen-reader support + reliably-tappable buttons app-wide</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>Parked fast-follow</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>a11y</t>
-        </is>
-      </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>PARTIAL</t>
-        </is>
-      </c>
-      <c r="G37" s="3" t="inlineStr">
-        <is>
-          <t>NW screens now labeled; rest of app partial</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>Roll the NW a11y pattern across all screens</t>
-        </is>
-      </c>
-      <c r="I37" s="3" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="J37" s="5" t="inlineStr"/>
-      <c r="K37" s="5" t="inlineStr"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>— D. PARKED V1 — launch blockers (see finwise-launch-and-parked.xlsx) —</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>P-41/P-39</t>
+          <t>L-1</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>UI/UX</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Undo-after-delete + skeleton loaders / offline-sync states</t>
+          <t>Switch to a paid/licensed price source (Tiingo). Free Yahoo feed isn't legal for a paid app</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Parked fast-follow</t>
+          <t>Parked V1</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>UX</t>
+          <t>Blocker</t>
         </is>
       </c>
       <c r="F38" s="6" t="inlineStr">
@@ -2187,17 +2187,17 @@
       </c>
       <c r="G38" s="3" t="inlineStr">
         <is>
-          <t>Not built</t>
+          <t>Seam ready; needs your API key</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr">
         <is>
-          <t>SEE PM REVIEW — part of the 'feels trustworthy' system</t>
+          <t>You get a key; I do the swap</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr"/>
@@ -2206,27 +2206,27 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>EXPAND</t>
+          <t>P-71</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>UI/UX</t>
+          <t>Branding</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Expand/collapse on long lists/sections (your example) — declutter every dense screen</t>
+          <t>Pick + trademark final app name ('FinWise' may be taken; 'Hatcho' front-runner)</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Your meta-feedback (this session)</t>
+          <t>Parked V1</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>UX system</t>
+          <t>Blocker</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
@@ -2236,21 +2236,479 @@
       </c>
       <c r="G39" s="3" t="inlineStr">
         <is>
-          <t>Not implemented anywhere</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>SEE PM REVIEW — build as a reusable pattern, apply to NW sections, budget buckets, holdings, insights</t>
+          <t>Decide name; then I do the rename pass (once, late)</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr"/>
       <c r="K39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>L-5..L-26</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Launch ops</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>App Store listing, privacy questionnaire, reviewer login, screenshots, build #35, submit</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Parked V1</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Blocker</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Your-owned; build #35 blocked on free EAS quota (~Jul 1)</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Sequence after the code is launch-ready</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr"/>
+      <c r="K40" s="5" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>P-23/P-63</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Dependency security scan + audit all data-fetch error handling (not just happy path)</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>Parked V1</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Important</t>
+        </is>
+      </c>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>I can do both before submit</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr"/>
+      <c r="K41" s="5" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>— E. PARKED — fast-follow &amp; V2 highlights (full list in parked xlsx) —</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>P-1</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>Bank/brokerage linking (auto-sync balances &amp; transactions)</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Parked V2</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Large build; needs secure server</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>SEE PM REVIEW — this is the #1 retention lever; reconsider priority</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr"/>
+      <c r="K43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>P-8</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Insights</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>'Can I afford a $600k house?' — plain-question affordability simulator</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Parked V2</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F44" s="6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Not built</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>SEE PM REVIEW — standout/shareable; move up</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr"/>
+      <c r="K44" s="5" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>P-35</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Home card: net worth over time ('up $40k in 6 months')</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Parked V2</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>Snapshot only today</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>SEE PM REVIEW — retention dopamine; move up</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr"/>
+      <c r="K45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>P-53</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Goals</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Finish the full savings-goals screen (progress, priority, projections)</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Parked fast-follow</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="F46" s="6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Logic exists; visual screen unfinished</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Good stickiness; pair with OPEN-3</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr"/>
+      <c r="K46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>P-28/P-29</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>a11y</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>Screen-reader support + reliably-tappable buttons app-wide</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Parked fast-follow</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>a11y</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>PARTIAL</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>NW screens now labeled; rest of app partial</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Roll the NW a11y pattern across all screens</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr"/>
+      <c r="K47" s="5" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>P-41/P-39</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Undo-after-delete + skeleton loaders / offline-sync states</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Parked fast-follow</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>UX</t>
+        </is>
+      </c>
+      <c r="F48" s="6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Not built</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>SEE PM REVIEW — part of the 'feels trustworthy' system</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr"/>
+      <c r="K48" s="5" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>EXPAND</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>UI/UX</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Expand/collapse on long lists/sections (your example) — declutter every dense screen</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Your meta-feedback (this session)</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>UX system</t>
+        </is>
+      </c>
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented anywhere</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>SEE PM REVIEW — build as a reusable pattern, apply to NW sections, budget buckets, holdings, insights</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr"/>
+      <c r="K49" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: add Phase 2 — Persona platform tab to master list
One platform, two switchable persona modes (Employed accumulation / Retired
decumulation) on a shared spine — NOT two separate apps. Architecture, screen split,
sequencing (Employed-first → Retired as 2nd surface → 50-65 glide path), and the gated
doc chain (PRD → conceptual → detailed → build). Approval/comments columns included.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-master-action-list-2026-06-28.xlsx
+++ b/docs/finwise-master-action-list-2026-06-28.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Master action list" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Principal PM review" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Phase 2 — Persona platform" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3120,4 +3121,600 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Decision / item</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Phase / sequencing</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>✅ Approve?</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>💬 Your comments</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="110" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>WHY</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>PHASE 2 — 'Money Command Center' as ONE platform serving two personas: Employed (18–55, accumulation) and Retired (decumulation). Decision: build as ONE platform with two switchable persona MODES sharing a common spine — NOT two separate apps. The spine (~70%: data model, net worth, holdings, taxonomy, security, prices, accuracy guarantees) is built once; the persona 'mode' swaps the Home dashboard, module set, planning lens, and tone. Sequence: ship Employed mode first → add Retired as the 2nd surface on the same spine → a 'glide path' for the 50–65 transition (the highest-value, semi-retired segment).</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="n"/>
+      <c r="D2" s="8" t="n"/>
+      <c r="E2" s="8" t="n"/>
+      <c r="F2" s="9" t="n"/>
+      <c r="G2" s="9" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>— ARCHITECTURE —</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>ONE platform, two switchable persona modes (NOT two separate softwares)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Forking into two apps = 2× maintenance, the cross-screen accuracy guarantees break across the fork, and you orphan the pre-retiree. One codebase, one subscription, one accuracy net.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Decision</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Shared spine — build once</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Auth, security/encryption, sync, the full data model (accounts, net worth, holdings, taxonomy, income, debts, transactions), market prices, most calculations + the agreement tests. ~70% of the work, identical for both personas.</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Foundation (largely built)</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr"/>
+      <c r="G5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Persona 'mode' layer — diverges</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Home dashboard (the hero question), the active module set, the planning lens (grow-toward vs draw-down), tone + onboarding questions, which insights fire.</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Per persona</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Mode chosen at onboarding; switchable</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Auto-suggest from age + employment/retirement status; user can switch. Stored on the profile.</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>With Employed mode</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>'Glide path' for the 50–65 transition</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Semi-retired / phasing users see BOTH lenses — still earning + starting to draw down. Highest-anxiety, highest-willingness-to-pay segment; the bridge competitors miss.</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>After both modes exist</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>— SCREEN SPLIT —</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Shared</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Auth · onboarding (persona fork early) · Net Worth · Investments/holdings · Settings · security.</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Spine</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Employed lens (accumulation)</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Home (on-track?) · Budget / cash-flow · Goals · Debt payoff · accumulation retirement projection · 'Can I afford X?'.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Mode 1 (first)</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr"/>
+      <c r="G11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Screens</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Retired lens (decumulation)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Home (will it last? safe-to-spend) · Withdrawal planner (required minimum withdrawals, Social Security timing, Roth conversions, draw sequencing) · healthcare/Medicare · odds-based drawdown projection · estate · tax-smart spend-down.</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Mode 2 (next surface)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>— SEQUENCING —</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Sequencing</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Ship Employed mode FIRST</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Mostly built, bigger market, faster to revenue. Focus the wedge here (18–35 start).</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Now</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sequencing</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Extract the shared spine AS you add Retired mode</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Don't speculatively architect a 'platform' before the 2nd mode proves the seams — premature abstraction = 2× complexity, ships nothing.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>When building mode 2</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Sequencing</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Retired mode = 2nd surface on the spine</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Not a parallel build. Reuse the spine; add the decumulation modules + lens.</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>After mode 1 ships</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Sequencing</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Do NOT build both pre-launch</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Scope discipline — nail one persona to revenue before the second.</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Guardrail</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>— PROCESS (doc chain, gated) —</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Product Requirements (PRD) per persona</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Persona + WEDGE + jobs-to-be-done + success metric + explicit scope cut (what's OUT). 2–3 pages. → YOU APPROVE before design.</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Gate 1</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Conceptual design</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Experience architecture, navigation model, key flows, how the wedge shows up. Mockup-level. → APPROVE before detail.</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Gate 2</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Detailed design (per screen/flow)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Layouts, states, components, copy, edge cases. → APPROVE before build.</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Gate 3</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Process</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Build → verify → device-test</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Each approved spec becomes code; gates stay green; verify on device.</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Gate 4</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>